<commit_message>
36 działajacych i przetestowanych umiejetności
</commit_message>
<xml_diff>
--- a/Dane/karty_v1.xlsx
+++ b/Dane/karty_v1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a40667ca9a5261e0/Dokumenty/Dokumenty/Gra Walka o Dusze/Symulator/Dane/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="116" documentId="8_{C60639C0-3DC1-46DF-8FF5-DD98044E12E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{80763C81-E1F9-420E-B8B9-DDA2F3FD6DC3}"/>
+  <xr:revisionPtr revIDLastSave="224" documentId="8_{C60639C0-3DC1-46DF-8FF5-DD98044E12E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{662FDB3F-4B7A-4C79-B4B9-EAB38EAF43D3}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1C612D17-AB6F-4FCE-AA6C-1D2201D34FB7}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Arkusz1!$A$1:$X$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Arkusz1!$A$1:$Z$98</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,6 +33,55 @@
     <author>Mariusz Janeczko</author>
   </authors>
   <commentList>
+    <comment ref="I1" authorId="0" shapeId="0" xr:uid="{F7200FBB-9721-4E27-803F-57F6C2399E04}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Mariusz Janeczko:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+musi być warunkowa 
+b- oznacza brak warunku</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="N12" authorId="0" shapeId="0" xr:uid="{9ED59B26-42DD-43C9-842D-3AE9CA821EE5}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Mariusz Janeczko:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+trzy użycia czyli wszyscy na arenie</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="H15" authorId="0" shapeId="0" xr:uid="{99EB7673-5FD0-4BC1-9BA0-E90A43A21D65}">
       <text>
         <r>
@@ -55,11 +104,35 @@
             <charset val="238"/>
           </rPr>
           <t xml:space="preserve">
-ZYCIE - zdolnosc nr 1 to ocalenie przeciwnika, dolnosc nr 2 to zabicie śmierci</t>
+ZYCIE - zdolnosc nr 1 to ocalenie przeciwnika</t>
         </r>
       </text>
     </comment>
-    <comment ref="H34" authorId="0" shapeId="0" xr:uid="{A6E5B52D-9858-4032-ADC8-5AB9224B7549}">
+    <comment ref="N29" authorId="0" shapeId="0" xr:uid="{3E0F4ED4-DC85-46A7-96AF-8D43B26507BE}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Mariusz Janeczko:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+1 użycie czyli tylko jeden sojusznik po tobie</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="H35" authorId="0" shapeId="0" xr:uid="{A6E5B52D-9858-4032-ADC8-5AB9224B7549}">
       <text>
         <r>
           <rPr>
@@ -90,7 +163,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="103">
   <si>
     <t>klasa</t>
   </si>
@@ -365,9 +438,6 @@
     <t>brak</t>
   </si>
   <si>
-    <t>F</t>
-  </si>
-  <si>
     <t>klasa_wroga&lt;</t>
   </si>
   <si>
@@ -384,13 +454,31 @@
   </si>
   <si>
     <t>b</t>
+  </si>
+  <si>
+    <t>ok all</t>
+  </si>
+  <si>
+    <t>2K2</t>
+  </si>
+  <si>
+    <t>klasa_wroga&lt;=</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>Duch Łaski</t>
+  </si>
+  <si>
+    <t>Terror</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
@@ -452,6 +540,43 @@
       <family val="2"/>
       <charset val="238"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="7"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="238"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0" tint="-4.9989318521683403E-2"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="238"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF6D6D"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="238"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -467,7 +592,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -490,11 +615,76 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF454545"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF454545"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF454545"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF454545"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF454545"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF454545"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF454545"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF454545"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF454545"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF454545"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF454545"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF454545"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF454545"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -512,6 +702,65 @@
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -877,10 +1126,10 @@
         <v>88</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>80</v>
@@ -949,6 +1198,9 @@
       </c>
       <c r="F2" s="2" t="s">
         <v>89</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>97</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>27</v>
@@ -996,7 +1248,7 @@
         <v>89</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H3" s="8" t="s">
         <v>27</v>
@@ -1054,7 +1306,7 @@
         <v>89</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H4" s="8" t="s">
         <v>27</v>
@@ -1112,7 +1364,7 @@
         <v>90</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H5" s="8" t="s">
         <v>54</v>
@@ -1121,7 +1373,9 @@
         <v>87</v>
       </c>
       <c r="J5" s="8"/>
-      <c r="K5" s="8"/>
+      <c r="K5" s="8" t="s">
+        <v>96</v>
+      </c>
       <c r="L5" s="8"/>
       <c r="M5" s="8"/>
       <c r="N5" s="8"/>
@@ -1168,7 +1422,7 @@
         <v>90</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="H6" s="8" t="s">
         <v>54</v>
@@ -1223,11 +1477,14 @@
       <c r="F7" s="2" t="s">
         <v>89</v>
       </c>
+      <c r="G7" s="2" t="s">
+        <v>95</v>
+      </c>
       <c r="H7" s="2" t="s">
         <v>27</v>
       </c>
       <c r="L7" s="2"/>
-      <c r="M7" s="2" t="s">
+      <c r="M7" s="9" t="s">
         <v>27</v>
       </c>
       <c r="N7" s="2" t="s">
@@ -1276,13 +1533,13 @@
       <c r="F8" s="2" t="s">
         <v>89</v>
       </c>
+      <c r="G8" s="2" t="s">
+        <v>95</v>
+      </c>
       <c r="H8" s="2" t="s">
         <v>27</v>
       </c>
       <c r="L8" s="2"/>
-      <c r="M8" s="2" t="s">
-        <v>21</v>
-      </c>
       <c r="N8" s="2" t="s">
         <v>21</v>
       </c>
@@ -1327,6 +1584,9 @@
       <c r="F9" s="2" t="s">
         <v>89</v>
       </c>
+      <c r="G9" s="2" t="s">
+        <v>95</v>
+      </c>
       <c r="H9" s="2" t="s">
         <v>27</v>
       </c>
@@ -1383,6 +1643,9 @@
       <c r="F10" s="2" t="s">
         <v>89</v>
       </c>
+      <c r="G10" s="2" t="s">
+        <v>95</v>
+      </c>
       <c r="H10" s="2" t="s">
         <v>27</v>
       </c>
@@ -1441,6 +1704,9 @@
       <c r="F11" s="2" t="s">
         <v>89</v>
       </c>
+      <c r="G11" s="2" t="s">
+        <v>95</v>
+      </c>
       <c r="H11" s="2" t="s">
         <v>27</v>
       </c>
@@ -1493,14 +1759,20 @@
       <c r="F12" s="2" t="s">
         <v>89</v>
       </c>
+      <c r="G12" s="2" t="s">
+        <v>95</v>
+      </c>
       <c r="H12" s="2" t="s">
         <v>27</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>87</v>
       </c>
+      <c r="K12" s="2" t="s">
+        <v>96</v>
+      </c>
       <c r="L12" s="2"/>
-      <c r="M12" s="4" t="s">
+      <c r="M12" s="8" t="s">
         <v>87</v>
       </c>
       <c r="N12" s="2" t="s">
@@ -1546,13 +1818,13 @@
       <c r="E13" s="2">
         <v>10</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="F13" s="13" t="s">
         <v>89</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="H13" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="H13" s="10" t="s">
         <v>27</v>
       </c>
       <c r="J13" s="2" t="s">
@@ -1596,17 +1868,20 @@
       <c r="E14" s="2">
         <v>11</v>
       </c>
-      <c r="F14" s="2" t="s">
-        <v>91</v>
+      <c r="F14" s="13" t="s">
+        <v>89</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>54</v>
+        <v>95</v>
+      </c>
+      <c r="H14" s="10" t="s">
+        <v>27</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>23</v>
+        <v>87</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>78</v>
       </c>
       <c r="L14" s="2" t="s">
         <v>23</v>
@@ -1653,11 +1928,14 @@
       <c r="E15" s="2">
         <v>12</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="F15" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="H15" s="2" t="s">
-        <v>23</v>
+      <c r="G15" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="H15" s="10" t="s">
+        <v>27</v>
       </c>
       <c r="L15" s="2"/>
       <c r="N15" s="2"/>
@@ -1699,15 +1977,20 @@
       <c r="E16" s="2">
         <v>13</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="F16" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="H16" s="2" t="s">
+      <c r="G16" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="H16" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="L16" s="2"/>
+      <c r="L16" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="M16" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="N16" s="2" t="s">
         <v>71</v>
@@ -1715,7 +1998,9 @@
       <c r="O16" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="P16" s="8"/>
+      <c r="P16" s="8" t="s">
+        <v>96</v>
+      </c>
       <c r="Q16" s="8" t="s">
         <v>7</v>
       </c>
@@ -1747,13 +2032,16 @@
       <c r="D17" s="2">
         <v>4</v>
       </c>
-      <c r="E17" s="2">
+      <c r="E17" s="8">
         <v>14</v>
       </c>
-      <c r="F17" s="2" t="s">
+      <c r="F17" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="H17" s="2" t="s">
+      <c r="G17" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="H17" s="10" t="s">
         <v>27</v>
       </c>
       <c r="I17" s="2" t="s">
@@ -1790,10 +2078,10 @@
       <c r="Z17" s="2"/>
     </row>
     <row r="18" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A18" s="2">
+      <c r="A18" s="8">
         <v>17</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="8" t="s">
         <v>30</v>
       </c>
       <c r="C18" s="2" t="s">
@@ -1802,13 +2090,16 @@
       <c r="D18" s="2">
         <v>5</v>
       </c>
-      <c r="E18" s="2">
+      <c r="E18" s="8">
         <v>13</v>
       </c>
-      <c r="F18" s="2" t="s">
+      <c r="F18" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="H18" s="2" t="s">
+      <c r="G18" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="H18" s="10" t="s">
         <v>27</v>
       </c>
       <c r="J18" s="2" t="s">
@@ -1840,10 +2131,10 @@
       <c r="Z18" s="2"/>
     </row>
     <row r="19" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A19" s="2">
+      <c r="A19" s="8">
         <v>18</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="8" t="s">
         <v>14</v>
       </c>
       <c r="C19" s="2" t="s">
@@ -1852,23 +2143,23 @@
       <c r="D19" s="2">
         <v>5</v>
       </c>
-      <c r="E19" s="2">
-        <v>15</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>91</v>
+      <c r="E19" s="26">
+        <v>16</v>
+      </c>
+      <c r="F19" s="13" t="s">
+        <v>90</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="H19" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="H19" s="10" t="s">
         <v>54</v>
       </c>
-      <c r="I19" s="2" t="s">
-        <v>15</v>
+      <c r="K19" s="2" t="s">
+        <v>96</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>15</v>
+        <v>98</v>
       </c>
       <c r="N19" s="2"/>
       <c r="O19" s="8" t="s">
@@ -1889,10 +2180,10 @@
       <c r="Z19" s="2"/>
     </row>
     <row r="20" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A20" s="2">
+      <c r="A20" s="8">
         <v>19</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="8" t="s">
         <v>3</v>
       </c>
       <c r="C20" s="2" t="s">
@@ -1901,17 +2192,14 @@
       <c r="D20" s="2">
         <v>5</v>
       </c>
-      <c r="E20" s="2">
+      <c r="E20" s="27">
         <v>99</v>
       </c>
-      <c r="F20" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="H20" s="2" t="s">
-        <v>54</v>
+      <c r="F20" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="H20" s="10" t="s">
+        <v>27</v>
       </c>
       <c r="L20" s="2"/>
       <c r="N20" s="2"/>
@@ -1935,163 +2223,136 @@
       <c r="Y20" s="2"/>
       <c r="Z20" s="2"/>
     </row>
-    <row r="21" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A21" s="2">
-        <v>1</v>
-      </c>
-      <c r="B21" s="2" t="s">
+    <row r="21" spans="1:26" s="19" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="22" t="s">
+        <v>100</v>
+      </c>
+      <c r="B21" s="22" t="s">
+        <v>101</v>
+      </c>
+      <c r="C21" s="19" t="s">
+        <v>4</v>
+      </c>
+      <c r="D21" s="29">
+        <v>4</v>
+      </c>
+      <c r="E21" s="28">
+        <v>12</v>
+      </c>
+      <c r="F21" s="20"/>
+      <c r="H21" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="N21" s="25"/>
+    </row>
+    <row r="22" spans="1:26" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="14">
+        <v>1</v>
+      </c>
+      <c r="B22" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C22" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="D21" s="2">
-        <v>1</v>
-      </c>
-      <c r="E21" s="2">
-        <v>1</v>
-      </c>
-      <c r="F21" s="2" t="s">
+      <c r="D22" s="14">
+        <v>1</v>
+      </c>
+      <c r="E22" s="18">
+        <v>1</v>
+      </c>
+      <c r="F22" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="H21" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L21" s="2"/>
-      <c r="N21" s="2" t="s">
+      <c r="G22" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="H22" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="I22" s="14"/>
+      <c r="J22" s="14"/>
+      <c r="K22" s="14"/>
+      <c r="L22" s="14"/>
+      <c r="M22" s="14"/>
+      <c r="N22" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="O21" s="8" t="s">
+      <c r="O22" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="P21" s="8"/>
-      <c r="Q21" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="T21" s="2">
+      <c r="P22" s="18"/>
+      <c r="Q22" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="R22" s="14"/>
+      <c r="S22" s="14"/>
+      <c r="T22" s="14">
         <v>0</v>
       </c>
-      <c r="W21" s="2" t="s">
+      <c r="U22" s="14"/>
+      <c r="V22" s="14"/>
+      <c r="W22" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="X21" s="2" t="s">
+      <c r="X22" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="Y21" s="2"/>
-      <c r="Z21" s="2"/>
-    </row>
-    <row r="22" spans="1:26" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="8">
+      <c r="Y22" s="14"/>
+      <c r="Z22" s="14"/>
+    </row>
+    <row r="23" spans="1:26" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="2">
         <v>2</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="B23" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C22" s="8" t="s">
+      <c r="C23" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D22" s="8">
-        <v>1</v>
-      </c>
-      <c r="E22" s="8">
+      <c r="D23" s="2">
+        <v>1</v>
+      </c>
+      <c r="E23" s="8">
         <v>2</v>
       </c>
-      <c r="F22" s="8" t="s">
+      <c r="F23" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="G22" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="H22" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="I22" s="8" t="s">
+      <c r="G23" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="H23" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I23" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="J22" s="8"/>
-      <c r="K22" s="8" t="s">
+      <c r="J23" s="8"/>
+      <c r="K23" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="L22" s="8"/>
-      <c r="M22" s="8"/>
-      <c r="N22" s="8"/>
-      <c r="O22" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="P22" s="8"/>
-      <c r="Q22" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="R22" s="8">
-        <v>1</v>
-      </c>
-      <c r="S22" s="8"/>
-      <c r="T22" s="8">
-        <v>1</v>
-      </c>
-      <c r="U22" s="8">
-        <v>1</v>
-      </c>
-      <c r="V22" s="8"/>
-      <c r="W22" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="X22" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="Y22" s="8"/>
-      <c r="Z22" s="8"/>
-    </row>
-    <row r="23" spans="1:26" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="8">
-        <v>3</v>
-      </c>
-      <c r="B23" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="C23" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="D23" s="8">
-        <v>1</v>
-      </c>
-      <c r="E23" s="8">
-        <v>3</v>
-      </c>
-      <c r="F23" s="8" t="s">
-        <v>89</v>
-      </c>
-      <c r="G23" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="H23" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="I23" s="8"/>
-      <c r="J23" s="8"/>
-      <c r="K23" s="8"/>
       <c r="L23" s="8"/>
-      <c r="M23" s="8">
-        <v>1</v>
-      </c>
-      <c r="N23" s="8" t="s">
-        <v>69</v>
-      </c>
+      <c r="M23" s="8"/>
+      <c r="N23" s="8"/>
       <c r="O23" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="P23" s="8" t="s">
-        <v>74</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="P23" s="8"/>
       <c r="Q23" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="R23" s="8"/>
+      <c r="R23" s="8">
+        <v>1</v>
+      </c>
       <c r="S23" s="8"/>
       <c r="T23" s="8">
-        <v>0</v>
-      </c>
-      <c r="U23" s="8"/>
+        <v>1</v>
+      </c>
+      <c r="U23" s="8">
+        <v>1</v>
+      </c>
       <c r="V23" s="8"/>
       <c r="W23" s="8" t="s">
         <v>11</v>
@@ -2103,43 +2364,45 @@
       <c r="Z23" s="8"/>
     </row>
     <row r="24" spans="1:26" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="8">
-        <v>4</v>
-      </c>
-      <c r="B24" s="8" t="s">
+      <c r="A24" s="2">
+        <v>3</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C24" s="8" t="s">
+      <c r="C24" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D24" s="8">
+      <c r="D24" s="2">
         <v>1</v>
       </c>
       <c r="E24" s="8">
-        <v>4</v>
-      </c>
-      <c r="F24" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="F24" s="16" t="s">
         <v>89</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="H24" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="H24" s="10" t="s">
         <v>27</v>
       </c>
       <c r="I24" s="8"/>
       <c r="J24" s="8"/>
       <c r="K24" s="8"/>
       <c r="L24" s="8"/>
-      <c r="M24" s="8"/>
+      <c r="M24" s="8">
+        <v>1</v>
+      </c>
       <c r="N24" s="8" t="s">
-        <v>86</v>
+        <v>69</v>
       </c>
       <c r="O24" s="8" t="s">
         <v>7</v>
       </c>
       <c r="P24" s="8" t="s">
-        <v>64</v>
+        <v>74</v>
       </c>
       <c r="Q24" s="8" t="s">
         <v>8</v>
@@ -2161,122 +2424,124 @@
       <c r="Z24" s="8"/>
     </row>
     <row r="25" spans="1:26" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="8">
-        <v>5</v>
-      </c>
-      <c r="B25" s="8" t="s">
+      <c r="A25" s="2">
+        <v>4</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C25" s="8" t="s">
+      <c r="C25" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D25" s="8">
-        <v>1</v>
-      </c>
-      <c r="E25" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="F25" s="8" t="s">
+      <c r="D25" s="2">
+        <v>1</v>
+      </c>
+      <c r="E25" s="8">
+        <v>4</v>
+      </c>
+      <c r="F25" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="G25" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="H25" s="8" t="s">
-        <v>23</v>
+      <c r="G25" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="H25" s="10" t="s">
+        <v>27</v>
       </c>
       <c r="I25" s="8"/>
-      <c r="J25" s="8" t="s">
-        <v>33</v>
-      </c>
+      <c r="J25" s="8"/>
       <c r="K25" s="8"/>
       <c r="L25" s="8"/>
       <c r="M25" s="8"/>
-      <c r="N25" s="8"/>
+      <c r="N25" s="8" t="s">
+        <v>86</v>
+      </c>
       <c r="O25" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="P25" s="8"/>
+        <v>7</v>
+      </c>
+      <c r="P25" s="8" t="s">
+        <v>64</v>
+      </c>
       <c r="Q25" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="R25" s="8">
-        <v>1</v>
-      </c>
+      <c r="R25" s="8"/>
       <c r="S25" s="8"/>
       <c r="T25" s="8">
-        <v>1</v>
-      </c>
-      <c r="U25" s="8">
-        <v>1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="U25" s="8"/>
       <c r="V25" s="8"/>
       <c r="W25" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="X25" s="8"/>
+      <c r="X25" s="8" t="s">
+        <v>18</v>
+      </c>
       <c r="Y25" s="8"/>
       <c r="Z25" s="8"/>
     </row>
-    <row r="26" spans="1:26" s="6" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:26" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>31</v>
       </c>
       <c r="D26" s="2">
-        <v>2</v>
-      </c>
-      <c r="E26" s="2">
-        <v>5</v>
-      </c>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
-      <c r="H26" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I26" s="2"/>
-      <c r="J26" s="2"/>
-      <c r="K26" s="2"/>
-      <c r="L26" s="2">
-        <v>1</v>
-      </c>
-      <c r="M26" s="2"/>
-      <c r="N26" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="E26" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F26" s="16" t="s">
+        <v>89</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="H26" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="I26" s="8"/>
+      <c r="J26" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="K26" s="8"/>
+      <c r="L26" s="8"/>
+      <c r="M26" s="8"/>
+      <c r="N26" s="8"/>
       <c r="O26" s="8" t="s">
         <v>8</v>
       </c>
       <c r="P26" s="8"/>
       <c r="Q26" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="R26" s="4">
-        <v>4</v>
-      </c>
-      <c r="S26" s="4"/>
-      <c r="T26" s="4">
-        <v>2</v>
-      </c>
-      <c r="U26" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="V26" s="4"/>
-      <c r="W26" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="X26" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="Y26" s="4"/>
-      <c r="Z26" s="4"/>
-    </row>
-    <row r="27" spans="1:26" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+      <c r="R26" s="8">
+        <v>1</v>
+      </c>
+      <c r="S26" s="8"/>
+      <c r="T26" s="8">
+        <v>1</v>
+      </c>
+      <c r="U26" s="8">
+        <v>1</v>
+      </c>
+      <c r="V26" s="8"/>
+      <c r="W26" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="X26" s="8"/>
+      <c r="Y26" s="8"/>
+      <c r="Z26" s="8"/>
+    </row>
+    <row r="27" spans="1:26" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>34</v>
@@ -2287,43 +2552,52 @@
       <c r="D27" s="2">
         <v>2</v>
       </c>
-      <c r="E27" s="2">
+      <c r="E27" s="8">
         <v>5</v>
       </c>
-      <c r="F27" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="G27" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="H27" s="2" t="s">
+      <c r="F27" s="13"/>
+      <c r="G27" s="2"/>
+      <c r="H27" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="I27" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="L27" s="2"/>
+      <c r="I27" s="2"/>
+      <c r="J27" s="2"/>
+      <c r="K27" s="2"/>
+      <c r="L27" s="2">
+        <v>1</v>
+      </c>
+      <c r="M27" s="2"/>
       <c r="N27" s="2"/>
       <c r="O27" s="8" t="s">
         <v>8</v>
       </c>
       <c r="P27" s="8"/>
       <c r="Q27" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="T27" s="2">
-        <v>0</v>
-      </c>
-      <c r="W27" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="X27" s="2"/>
-      <c r="Y27" s="2"/>
-      <c r="Z27" s="2"/>
+        <v>7</v>
+      </c>
+      <c r="R27" s="8">
+        <v>4</v>
+      </c>
+      <c r="S27" s="8"/>
+      <c r="T27" s="8">
+        <v>2</v>
+      </c>
+      <c r="U27" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="V27" s="8"/>
+      <c r="W27" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="X27" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="Y27" s="4"/>
+      <c r="Z27" s="4"/>
     </row>
     <row r="28" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>34</v>
@@ -2334,52 +2608,46 @@
       <c r="D28" s="2">
         <v>2</v>
       </c>
-      <c r="E28" s="2">
-        <v>6</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>27</v>
+      <c r="E28" s="8">
+        <v>5</v>
+      </c>
+      <c r="F28" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="H28" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="K28" s="2" t="s">
+        <v>96</v>
       </c>
       <c r="L28" s="2"/>
-      <c r="M28" s="2">
-        <v>3</v>
-      </c>
-      <c r="N28" s="2">
-        <v>1</v>
-      </c>
+      <c r="N28" s="2"/>
       <c r="O28" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="P28" s="8" t="s">
-        <v>37</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="P28" s="8"/>
       <c r="Q28" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="S28" s="2">
-        <v>1</v>
-      </c>
       <c r="T28" s="2">
-        <v>1</v>
-      </c>
-      <c r="U28" s="2" t="s">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="W28" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="X28" s="8" t="s">
-        <v>24</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="X28" s="2"/>
       <c r="Y28" s="2"/>
       <c r="Z28" s="2"/>
     </row>
     <row r="29" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>34</v>
@@ -2390,50 +2658,55 @@
       <c r="D29" s="2">
         <v>2</v>
       </c>
-      <c r="E29" s="2">
-        <v>7</v>
-      </c>
-      <c r="F29" s="2" t="s">
+      <c r="E29" s="8">
+        <v>6</v>
+      </c>
+      <c r="F29" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="H29" s="2" t="s">
+      <c r="G29" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="H29" s="10" t="s">
         <v>27</v>
       </c>
       <c r="L29" s="2"/>
       <c r="M29" s="2">
-        <v>2</v>
-      </c>
-      <c r="N29" s="2" t="s">
-        <v>69</v>
+        <v>3</v>
+      </c>
+      <c r="N29" s="2">
+        <v>1</v>
       </c>
       <c r="O29" s="8" t="s">
         <v>7</v>
       </c>
       <c r="P29" s="8" t="s">
-        <v>74</v>
+        <v>37</v>
       </c>
       <c r="Q29" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="S29" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="T29" s="2" t="s">
-        <v>27</v>
+      <c r="S29" s="2">
+        <v>1</v>
+      </c>
+      <c r="T29" s="2">
+        <v>1</v>
       </c>
       <c r="U29" s="2" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="W29" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="X29" s="8"/>
+        <v>12</v>
+      </c>
+      <c r="X29" s="8" t="s">
+        <v>24</v>
+      </c>
       <c r="Y29" s="2"/>
       <c r="Z29" s="2"/>
     </row>
     <row r="30" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>34</v>
@@ -2444,108 +2717,111 @@
       <c r="D30" s="2">
         <v>2</v>
       </c>
-      <c r="E30" s="2">
-        <v>8</v>
-      </c>
-      <c r="F30" s="2" t="s">
+      <c r="E30" s="8">
+        <v>7</v>
+      </c>
+      <c r="F30" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="H30" s="2" t="s">
-        <v>23</v>
+      <c r="G30" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="H30" s="10" t="s">
+        <v>27</v>
       </c>
       <c r="L30" s="2"/>
       <c r="M30" s="2">
-        <v>3.1</v>
+        <v>2</v>
       </c>
       <c r="N30" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="O30" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="P30" s="8"/>
+      <c r="P30" s="8" t="s">
+        <v>74</v>
+      </c>
       <c r="Q30" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="R30" s="2">
-        <v>1</v>
-      </c>
       <c r="S30" s="2" t="s">
-        <v>61</v>
+        <v>27</v>
       </c>
       <c r="T30" s="2" t="s">
-        <v>51</v>
+        <v>27</v>
       </c>
       <c r="U30" s="2" t="s">
-        <v>60</v>
+        <v>23</v>
       </c>
       <c r="W30" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="X30" s="8" t="s">
-        <v>81</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="X30" s="8"/>
       <c r="Y30" s="2"/>
       <c r="Z30" s="2"/>
     </row>
     <row r="31" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>31</v>
       </c>
       <c r="D31" s="2">
-        <v>3</v>
-      </c>
-      <c r="E31" s="2">
-        <v>9</v>
-      </c>
-      <c r="F31" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E31" s="8">
+        <v>8</v>
+      </c>
+      <c r="F31" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="H31" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="I31" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="J31" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="K31" s="2" t="s">
-        <v>92</v>
+      <c r="G31" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="H31" s="10" t="s">
+        <v>27</v>
       </c>
       <c r="L31" s="2"/>
-      <c r="N31" s="2"/>
+      <c r="M31" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="N31" s="2" t="s">
+        <v>69</v>
+      </c>
       <c r="O31" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="P31" s="8"/>
+        <v>7</v>
+      </c>
+      <c r="P31" s="8" t="s">
+        <v>75</v>
+      </c>
       <c r="Q31" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="T31" s="2">
-        <v>0</v>
+      <c r="S31" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="T31" s="8" t="s">
+        <v>27</v>
       </c>
       <c r="U31" s="2" t="s">
-        <v>27</v>
-      </c>
+        <v>59</v>
+      </c>
+      <c r="V31" s="3"/>
       <c r="W31" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="X31" s="8" t="s">
-        <v>18</v>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="X31" s="8"/>
       <c r="Y31" s="2"/>
       <c r="Z31" s="2"/>
     </row>
     <row r="32" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A32" s="2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>38</v>
@@ -2556,51 +2832,48 @@
       <c r="D32" s="2">
         <v>3</v>
       </c>
-      <c r="E32" s="2">
+      <c r="E32" s="8">
+        <v>9</v>
+      </c>
+      <c r="F32" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="H32" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="J32" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="L32" s="2"/>
+      <c r="N32" s="2"/>
+      <c r="O32" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="P32" s="8"/>
+      <c r="Q32" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="T32" s="2">
+        <v>0</v>
+      </c>
+      <c r="U32" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="W32" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="F32" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="H32" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L32" s="2"/>
-      <c r="M32" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="N32" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="O32" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="P32" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="Q32" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="S32" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="T32" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="U32" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="V32" s="3"/>
-      <c r="W32" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="X32" s="8"/>
+      <c r="X32" s="8" t="s">
+        <v>18</v>
+      </c>
       <c r="Y32" s="2"/>
       <c r="Z32" s="2"/>
     </row>
     <row r="33" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A33" s="2">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>38</v>
@@ -2611,97 +2884,107 @@
       <c r="D33" s="2">
         <v>3</v>
       </c>
-      <c r="E33" s="2">
-        <v>11</v>
-      </c>
-      <c r="F33" s="2" t="s">
-        <v>91</v>
+      <c r="E33" s="8">
+        <v>10</v>
+      </c>
+      <c r="F33" s="13" t="s">
+        <v>89</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="H33" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="I33" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="H33" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="L33" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="N33" s="2"/>
+      <c r="L33" s="2"/>
+      <c r="M33" s="2">
+        <v>3.1</v>
+      </c>
+      <c r="N33" s="2" t="s">
+        <v>71</v>
+      </c>
       <c r="O33" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="P33" s="8"/>
+        <v>7</v>
+      </c>
+      <c r="P33" s="2" t="s">
+        <v>99</v>
+      </c>
       <c r="Q33" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="T33" s="2">
-        <v>0</v>
-      </c>
-      <c r="W33" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="X33" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="Y33" s="2"/>
-      <c r="Z33" s="2"/>
+        <v>8</v>
+      </c>
+      <c r="R33" s="2">
+        <v>1</v>
+      </c>
+      <c r="S33" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="T33" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="U33" s="2" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="34" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A34" s="2">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C34" s="2" t="s">
         <v>31</v>
       </c>
       <c r="D34" s="2">
-        <v>4</v>
-      </c>
-      <c r="E34" s="2">
-        <v>12</v>
-      </c>
-      <c r="F34" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E34" s="8">
+        <v>11</v>
+      </c>
+      <c r="F34" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="H34" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L34" s="2"/>
+      <c r="G34" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="H34" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="K34" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="L34" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="N34" s="2"/>
       <c r="O34" s="8" t="s">
         <v>8</v>
       </c>
       <c r="P34" s="8"/>
       <c r="Q34" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="R34" s="2" t="s">
-        <v>58</v>
+        <v>7</v>
       </c>
       <c r="T34" s="2">
         <v>0</v>
       </c>
-      <c r="U34" s="2">
-        <v>1</v>
-      </c>
       <c r="W34" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="X34" s="8"/>
+        <v>11</v>
+      </c>
+      <c r="X34" s="8" t="s">
+        <v>24</v>
+      </c>
       <c r="Y34" s="2"/>
       <c r="Z34" s="2"/>
     </row>
     <row r="35" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A35" s="2">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>31</v>
@@ -2709,17 +2992,17 @@
       <c r="D35" s="2">
         <v>4</v>
       </c>
-      <c r="E35" s="2">
-        <v>13</v>
-      </c>
-      <c r="F35" s="2" t="s">
+      <c r="E35" s="8">
+        <v>12</v>
+      </c>
+      <c r="F35" s="13" t="s">
         <v>89</v>
       </c>
+      <c r="G35" s="2" t="s">
+        <v>95</v>
+      </c>
       <c r="H35" s="2" t="s">
         <v>27</v>
-      </c>
-      <c r="J35" s="2" t="s">
-        <v>43</v>
       </c>
       <c r="L35" s="2"/>
       <c r="N35" s="2"/>
@@ -2730,14 +3013,17 @@
       <c r="Q35" s="8" t="s">
         <v>8</v>
       </c>
+      <c r="R35" s="2" t="s">
+        <v>58</v>
+      </c>
       <c r="T35" s="2">
-        <v>1</v>
-      </c>
-      <c r="U35" s="2" t="s">
-        <v>27</v>
+        <v>0</v>
+      </c>
+      <c r="U35" s="2">
+        <v>1</v>
       </c>
       <c r="W35" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="X35" s="8"/>
       <c r="Y35" s="2"/>
@@ -2745,10 +3031,10 @@
     </row>
     <row r="36" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>31</v>
@@ -2756,36 +3042,32 @@
       <c r="D36" s="2">
         <v>4</v>
       </c>
-      <c r="E36" s="2">
-        <v>14</v>
-      </c>
-      <c r="F36" s="2" t="s">
+      <c r="E36" s="8">
+        <v>13</v>
+      </c>
+      <c r="F36" s="13" t="s">
         <v>89</v>
       </c>
+      <c r="G36" s="2" t="s">
+        <v>95</v>
+      </c>
       <c r="H36" s="2" t="s">
         <v>27</v>
       </c>
+      <c r="J36" s="2" t="s">
+        <v>43</v>
+      </c>
       <c r="L36" s="2"/>
-      <c r="M36" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="N36" s="2" t="s">
-        <v>69</v>
-      </c>
+      <c r="N36" s="2"/>
       <c r="O36" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="P36" s="8" t="s">
-        <v>73</v>
-      </c>
+        <v>8</v>
+      </c>
+      <c r="P36" s="8"/>
       <c r="Q36" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="S36" s="2">
-        <v>4</v>
-      </c>
       <c r="T36" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U36" s="2" t="s">
         <v>27</v>
@@ -2799,42 +3081,50 @@
     </row>
     <row r="37" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A37" s="2">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>31</v>
       </c>
       <c r="D37" s="2">
-        <v>5</v>
-      </c>
-      <c r="E37" s="2">
-        <v>13</v>
-      </c>
-      <c r="F37" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E37" s="8">
+        <v>14</v>
+      </c>
+      <c r="F37" s="13" t="s">
         <v>89</v>
       </c>
+      <c r="G37" s="2" t="s">
+        <v>95</v>
+      </c>
       <c r="H37" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="J37" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="L37" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="N37" s="2"/>
+      <c r="L37" s="2"/>
+      <c r="M37" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N37" s="2" t="s">
+        <v>69</v>
+      </c>
       <c r="O37" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="P37" s="8"/>
+        <v>7</v>
+      </c>
+      <c r="P37" s="8" t="s">
+        <v>73</v>
+      </c>
       <c r="Q37" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="T37" s="8">
-        <v>1</v>
+        <v>8</v>
+      </c>
+      <c r="S37" s="2">
+        <v>4</v>
+      </c>
+      <c r="T37" s="2">
+        <v>2</v>
       </c>
       <c r="U37" s="2" t="s">
         <v>27</v>
@@ -2842,18 +3132,16 @@
       <c r="W37" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="X37" s="8" t="s">
-        <v>24</v>
-      </c>
+      <c r="X37" s="8"/>
       <c r="Y37" s="2"/>
       <c r="Z37" s="2"/>
     </row>
     <row r="38" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A38" s="2">
-        <v>18</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>46</v>
+      <c r="A38" s="8">
+        <v>17</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>44</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>31</v>
@@ -2861,42 +3149,53 @@
       <c r="D38" s="2">
         <v>5</v>
       </c>
-      <c r="E38" s="2">
+      <c r="E38" s="8">
         <v>13</v>
       </c>
+      <c r="F38" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>95</v>
+      </c>
       <c r="H38" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="L38" s="2"/>
+      <c r="J38" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="L38" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="N38" s="2"/>
       <c r="O38" s="8" t="s">
         <v>8</v>
       </c>
       <c r="P38" s="8"/>
       <c r="Q38" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="T38" s="2">
-        <v>0</v>
+        <v>7</v>
+      </c>
+      <c r="T38" s="8">
+        <v>1</v>
       </c>
       <c r="U38" s="2" t="s">
         <v>27</v>
       </c>
       <c r="W38" s="2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="X38" s="8" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="Y38" s="2"/>
       <c r="Z38" s="2"/>
     </row>
     <row r="39" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="A39" s="2">
-        <v>19</v>
-      </c>
-      <c r="B39" s="2" t="s">
-        <v>47</v>
+      <c r="A39" s="8">
+        <v>18</v>
+      </c>
+      <c r="B39" s="8" t="s">
+        <v>46</v>
       </c>
       <c r="C39" s="2" t="s">
         <v>31</v>
@@ -2904,82 +3203,133 @@
       <c r="D39" s="2">
         <v>5</v>
       </c>
-      <c r="E39" s="2">
-        <v>15</v>
-      </c>
+      <c r="E39" s="27">
+        <v>13</v>
+      </c>
+      <c r="F39" s="13"/>
       <c r="H39" s="2" t="s">
         <v>27</v>
       </c>
       <c r="L39" s="2"/>
-      <c r="N39" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="O39" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="P39" s="2"/>
-      <c r="Q39" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="S39" s="3">
-        <v>3</v>
+      <c r="N39" s="2"/>
+      <c r="O39" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="P39" s="8"/>
+      <c r="Q39" s="8" t="s">
+        <v>8</v>
       </c>
       <c r="T39" s="2">
         <v>0</v>
       </c>
-      <c r="U39" s="2">
-        <v>1</v>
+      <c r="U39" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="W39" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="X39" s="8"/>
+      <c r="X39" s="8" t="s">
+        <v>18</v>
+      </c>
       <c r="Y39" s="2"/>
       <c r="Z39" s="2"/>
     </row>
     <row r="40" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="D40" s="1"/>
-      <c r="E40" s="1"/>
-      <c r="F40" s="1"/>
-      <c r="G40" s="1"/>
-      <c r="H40" s="1"/>
-      <c r="I40" s="1"/>
-      <c r="J40" s="1"/>
-      <c r="K40" s="1"/>
-      <c r="M40" s="1"/>
-      <c r="N40" s="1"/>
-      <c r="X40" s="7"/>
-    </row>
-    <row r="41" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="D41" s="1"/>
-      <c r="E41" s="1"/>
-      <c r="F41" s="1"/>
-      <c r="G41" s="1"/>
-      <c r="H41" s="1"/>
-      <c r="I41" s="1"/>
-      <c r="J41" s="1"/>
-      <c r="K41" s="1"/>
-      <c r="M41" s="1"/>
-      <c r="N41" s="1"/>
-      <c r="X41" s="7"/>
-    </row>
-    <row r="42" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="D42" s="1"/>
-      <c r="E42" s="1"/>
-      <c r="F42" s="1"/>
-      <c r="G42" s="1"/>
-      <c r="H42" s="1"/>
-      <c r="I42" s="1"/>
-      <c r="J42" s="1"/>
-      <c r="K42" s="1"/>
-      <c r="M42" s="1"/>
-      <c r="N42" s="1"/>
-      <c r="X42" s="7"/>
+      <c r="A40" s="8">
+        <v>19</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D40" s="2">
+        <v>5</v>
+      </c>
+      <c r="E40" s="27">
+        <v>15</v>
+      </c>
+      <c r="F40" s="13"/>
+      <c r="H40" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="L40" s="2"/>
+      <c r="N40" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="O40" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="P40" s="2"/>
+      <c r="Q40" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="S40" s="3">
+        <v>3</v>
+      </c>
+      <c r="T40" s="2">
+        <v>0</v>
+      </c>
+      <c r="U40" s="2">
+        <v>1</v>
+      </c>
+      <c r="W40" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="X40" s="8"/>
+      <c r="Y40" s="2"/>
+      <c r="Z40" s="2"/>
+    </row>
+    <row r="41" spans="1:26" s="19" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="22" t="s">
+        <v>100</v>
+      </c>
+      <c r="B41" s="22" t="s">
+        <v>102</v>
+      </c>
+      <c r="C41" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="D41" s="29">
+        <v>4</v>
+      </c>
+      <c r="E41" s="28">
+        <v>14</v>
+      </c>
+      <c r="F41" s="20"/>
+      <c r="H41" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="X41" s="22"/>
+    </row>
+    <row r="42" spans="1:26" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="F42" s="14"/>
+      <c r="G42" s="14"/>
+      <c r="H42" s="14"/>
+      <c r="I42" s="14"/>
+      <c r="J42" s="14"/>
+      <c r="K42" s="14"/>
+      <c r="M42" s="14"/>
+      <c r="N42" s="17"/>
+      <c r="R42" s="14"/>
+      <c r="S42" s="14"/>
+      <c r="T42" s="14"/>
+      <c r="U42" s="14"/>
+      <c r="V42" s="14"/>
+      <c r="W42" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="X42" s="18" t="s">
+        <v>81</v>
+      </c>
+      <c r="Y42" s="14"/>
+      <c r="Z42" s="14"/>
     </row>
     <row r="43" spans="1:26" x14ac:dyDescent="0.25">
       <c r="D43" s="1"/>
       <c r="E43" s="1"/>
-      <c r="F43" s="1"/>
+      <c r="F43" s="12"/>
       <c r="G43" s="1"/>
       <c r="H43" s="1"/>
       <c r="I43" s="1"/>
@@ -2992,7 +3342,7 @@
     <row r="44" spans="1:26" x14ac:dyDescent="0.25">
       <c r="D44" s="1"/>
       <c r="E44" s="1"/>
-      <c r="F44" s="1"/>
+      <c r="F44" s="12"/>
       <c r="G44" s="1"/>
       <c r="H44" s="1"/>
       <c r="I44" s="1"/>
@@ -3004,7 +3354,7 @@
     <row r="45" spans="1:26" x14ac:dyDescent="0.25">
       <c r="D45" s="1"/>
       <c r="E45" s="1"/>
-      <c r="F45" s="1"/>
+      <c r="F45" s="12"/>
       <c r="G45" s="1"/>
       <c r="H45" s="1"/>
       <c r="I45" s="1"/>
@@ -3016,7 +3366,7 @@
     <row r="46" spans="1:26" x14ac:dyDescent="0.25">
       <c r="D46" s="1"/>
       <c r="E46" s="1"/>
-      <c r="F46" s="1"/>
+      <c r="F46" s="12"/>
       <c r="G46" s="1"/>
       <c r="H46" s="1"/>
       <c r="I46" s="1"/>
@@ -3650,9 +4000,10 @@
       <c r="N98" s="1"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B21:X39">
-    <sortCondition ref="D21:D39"/>
-    <sortCondition ref="E21:E39"/>
+  <autoFilter ref="A1:Z98" xr:uid="{E5603586-01B1-45C3-888E-EC2BF5D85650}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B22:X40">
+    <sortCondition ref="D22:D40"/>
+    <sortCondition ref="E22:E40"/>
   </sortState>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>